<commit_message>
Verify Overview task visibility after employee starts work
</commit_message>
<xml_diff>
--- a/docs/qa40-results.xlsx
+++ b/docs/qa40-results.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" r:id="Rd68bedb049e04924"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case details" sheetId="2" r:id="Rbac9ddd1135447e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL comparison" sheetId="3" r:id="Rdc3131acd7044de8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" r:id="R2508f98eacaa4a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case details" sheetId="2" r:id="R1416152d63894d0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL comparison" sheetId="3" r:id="R8d70959d0633428f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -149,18 +149,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF7F6000"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF2CC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
+  <x:dxfs count="1">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -454,8 +443,8 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="1" t="str">
-        <x:f>"PASS: "&amp;COUNTIFS(B9:B48,"PASS")&amp;". FAIL: "&amp;COUNTIFS(B9:B48,"FAIL")&amp;". BLOCKED: "&amp;COUNTIFS(B9:B48,"BLOCKED")&amp;"."</x:f>
-        <x:v>PASS: 39. FAIL: 0. BLOCKED: 1.</x:v>
+        <x:f>"PASS: "&amp;COUNTIFS(B9:B48,"PASS")&amp;". FAIL: "&amp;COUNTIFS(B9:B48,"FAIL")&amp;"."</x:f>
+        <x:v>PASS: 40. FAIL: 0.</x:v>
       </x:c>
       <x:c r="B5" s="1"/>
       <x:c r="C5" s="1"/>
@@ -1474,35 +1463,36 @@
 1 screenshots</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="150.75" customHeight="1">
+    <x:row r="47" ht="125.25" customHeight="1">
       <x:c r="A47" s="10" t="str">
         <x:v>M39</x:v>
       </x:c>
       <x:c r="B47" s="10" t="str">
-        <x:v>BLOCKED</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="C47" s="10" t="str">
-        <x:v>R04,R07</x:v>
+        <x:v>R02,R04,R05,R10</x:v>
       </x:c>
       <x:c r="D47" s="10" t="str">
-        <x:v>Keyboard, desktop zoom, numeric alignment and saving feedback</x:v>
+        <x:v>Overview visibility before and after Employee starts a task</x:v>
       </x:c>
       <x:c r="E47" s="10" t="str">
-        <x:v>Controls reachable with visible focus, readable at 200%, and one save.</x:v>
+        <x:v>Admin/Manager totals include the project; TODO task appears in Work in progress only after Start task; Employee sees own TODO work; foreign Manager excluded.</x:v>
       </x:c>
       <x:c r="F47" s="10" t="str">
-        <x:v>Keyboard focus has visible outline
-Zoom-equivalent viewport has no page-level horizontal overflow
-Minutes has associated helper text
-Submit marks form busy and shows saving feedback
-Disabled button ignores a second click
-One entry saved through browser submission
-Time durations are right aligned
-Native browser 200% zoom and human usability assessment not executed. Zoom-equivalent reflow, keyboard and saving checks executed.</x:v>
+        <x:v>neha: TODO task excluded from Work in progress
+neha: new project included in summary
+admin: TODO task excluded from Work in progress
+admin: new project included in summary
+Employee Overview includes own TODO task
+Employee Start task button persists IN_PROGRESS
+neha: started task and project visible in Work in progress
+admin: started task and project visible in Work in progress
+Foreign Manager cannot see the task</x:v>
       </x:c>
       <x:c r="G47" s="10" t="str">
         <x:v>M39.json
-4 screenshots</x:v>
+5 screenshots</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
@@ -1532,12 +1522,11 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="B9:B48">
-    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="BLOCKED"/>
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="FAIL"/>
+    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FAIL"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9ef97027541434a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62d3a43cfc3944cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1665,7 +1654,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M2" s="14" t="d">
-        <x:v>2026-10-09T06:34:45.054Z</x:v>
+        <x:v>2026-10-09T08:36:51.469Z</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="210" customHeight="1">
@@ -1722,7 +1711,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M3" s="14" t="d">
-        <x:v>2026-10-09T06:34:48.663Z</x:v>
+        <x:v>2026-10-09T08:36:55.065Z</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="483" customHeight="1">
@@ -1801,7 +1790,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M4" s="14" t="d">
-        <x:v>2026-10-09T06:34:51.735Z</x:v>
+        <x:v>2026-10-09T08:36:57.992Z</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="210" customHeight="1">
@@ -1854,7 +1843,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M5" s="14" t="d">
-        <x:v>2026-10-09T06:34:56.162Z</x:v>
+        <x:v>2026-10-09T08:37:02.416Z</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="357" customHeight="1">
@@ -1921,7 +1910,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M6" s="14" t="d">
-        <x:v>2026-10-09T06:34:58.918Z</x:v>
+        <x:v>2026-10-09T08:37:05.171Z</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="315" customHeight="1">
@@ -1984,7 +1973,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M7" s="14" t="d">
-        <x:v>2026-10-09T06:35:02.179Z</x:v>
+        <x:v>2026-10-09T08:37:08.432Z</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="189" customHeight="1">
@@ -2039,7 +2028,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M8" s="14" t="d">
-        <x:v>2026-10-09T06:35:05.726Z</x:v>
+        <x:v>2026-10-09T08:37:11.929Z</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="315" customHeight="1">
@@ -2102,7 +2091,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M9" s="14" t="d">
-        <x:v>2026-10-09T06:35:08.861Z</x:v>
+        <x:v>2026-10-09T08:37:15.049Z</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="420" customHeight="1">
@@ -2173,7 +2162,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M10" s="14" t="d">
-        <x:v>2026-10-09T06:35:12.227Z</x:v>
+        <x:v>2026-10-09T08:37:18.417Z</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="672" customHeight="1">
@@ -2270,7 +2259,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M11" s="14" t="d">
-        <x:v>2026-10-09T06:35:15.583Z</x:v>
+        <x:v>2026-10-09T08:37:21.784Z</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="336" customHeight="1">
@@ -2332,7 +2321,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M12" s="14" t="d">
-        <x:v>2026-10-09T06:35:19.080Z</x:v>
+        <x:v>2026-10-09T08:37:25.215Z</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="546" customHeight="1">
@@ -2406,7 +2395,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M13" s="14" t="d">
-        <x:v>2026-10-09T06:35:22.351Z</x:v>
+        <x:v>2026-10-09T08:37:28.458Z</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="189" customHeight="1">
@@ -2459,7 +2448,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M14" s="14" t="d">
-        <x:v>2026-10-09T06:35:25.980Z</x:v>
+        <x:v>2026-10-09T08:37:32.109Z</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="126" customHeight="1">
@@ -2508,7 +2497,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M15" s="14" t="d">
-        <x:v>2026-10-09T06:35:28.809Z</x:v>
+        <x:v>2026-10-09T08:37:34.913Z</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="147" customHeight="1">
@@ -2557,7 +2546,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M16" s="14" t="d">
-        <x:v>2026-10-09T06:35:31.422Z</x:v>
+        <x:v>2026-10-09T08:37:37.510Z</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="336" customHeight="1">
@@ -2621,7 +2610,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M17" s="14" t="d">
-        <x:v>2026-10-09T06:35:34.178Z</x:v>
+        <x:v>2026-10-09T08:37:40.260Z</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="315" customHeight="1">
@@ -2681,7 +2670,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M18" s="14" t="d">
-        <x:v>2026-10-09T06:35:37.249Z</x:v>
+        <x:v>2026-10-09T08:37:43.369Z</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="210" customHeight="1">
@@ -2736,7 +2725,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M19" s="14" t="d">
-        <x:v>2026-10-09T06:35:40.516Z</x:v>
+        <x:v>2026-10-09T08:37:46.617Z</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="210" customHeight="1">
@@ -2791,7 +2780,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M20" s="14" t="d">
-        <x:v>2026-10-09T06:35:43.382Z</x:v>
+        <x:v>2026-10-09T08:37:49.493Z</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="147" customHeight="1">
@@ -2840,7 +2829,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M21" s="14" t="d">
-        <x:v>2026-10-09T06:35:46.225Z</x:v>
+        <x:v>2026-10-09T08:37:52.321Z</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="168" customHeight="1">
@@ -2893,7 +2882,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M22" s="14" t="d">
-        <x:v>2026-10-09T06:35:49.255Z</x:v>
+        <x:v>2026-10-09T08:37:55.193Z</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="168" customHeight="1">
@@ -2945,7 +2934,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M23" s="14" t="d">
-        <x:v>2026-10-09T06:35:51.991Z</x:v>
+        <x:v>2026-10-09T08:37:57.898Z</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="567" customHeight="1">
@@ -3027,7 +3016,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M24" s="14" t="d">
-        <x:v>2026-10-09T06:35:54.980Z</x:v>
+        <x:v>2026-10-09T08:38:00.912Z</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="483" customHeight="1">
@@ -3106,7 +3095,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M25" s="14" t="d">
-        <x:v>2026-10-09T06:35:58.463Z</x:v>
+        <x:v>2026-10-09T08:38:04.393Z</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="1113" customHeight="1">
@@ -3239,7 +3228,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M26" s="14" t="d">
-        <x:v>2026-10-09T06:36:01.746Z</x:v>
+        <x:v>2026-10-09T08:38:07.600Z</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="273" customHeight="1">
@@ -3300,7 +3289,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M27" s="14" t="d">
-        <x:v>2026-10-09T06:36:05.830Z</x:v>
+        <x:v>2026-10-09T08:38:11.648Z</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="378" customHeight="1">
@@ -3370,7 +3359,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M28" s="14" t="d">
-        <x:v>2026-10-09T06:36:08.836Z</x:v>
+        <x:v>2026-10-09T08:38:14.567Z</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="462" customHeight="1">
@@ -3445,7 +3434,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M29" s="14" t="d">
-        <x:v>2026-10-09T06:36:12.219Z</x:v>
+        <x:v>2026-10-09T08:38:17.938Z</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="609" customHeight="1">
@@ -3535,7 +3524,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M30" s="14" t="d">
-        <x:v>2026-10-09T06:36:15.661Z</x:v>
+        <x:v>2026-10-09T08:38:21.400Z</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="672" customHeight="1">
@@ -3629,7 +3618,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M31" s="14" t="d">
-        <x:v>2026-10-09T06:36:19.798Z</x:v>
+        <x:v>2026-10-09T08:38:25.507Z</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="567" customHeight="1">
@@ -3714,7 +3703,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M32" s="14" t="d">
-        <x:v>2026-10-09T06:36:23.575Z</x:v>
+        <x:v>2026-10-09T08:38:29.275Z</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="273" customHeight="1">
@@ -3773,7 +3762,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M33" s="14" t="d">
-        <x:v>2026-10-09T06:36:27.004Z</x:v>
+        <x:v>2026-10-09T08:38:32.690Z</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="273" customHeight="1">
@@ -3831,7 +3820,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M34" s="14" t="d">
-        <x:v>2026-10-09T06:36:29.986Z</x:v>
+        <x:v>2026-10-09T08:38:35.711Z</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="588" customHeight="1">
@@ -3917,7 +3906,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M35" s="14" t="d">
-        <x:v>2026-10-09T06:36:33.095Z</x:v>
+        <x:v>2026-10-09T08:38:38.935Z</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="525" customHeight="1">
@@ -3998,7 +3987,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M36" s="14" t="d">
-        <x:v>2026-10-09T06:36:36.669Z</x:v>
+        <x:v>2026-10-09T08:38:42.528Z</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="1197" customHeight="1">
@@ -4131,7 +4120,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M37" s="14" t="d">
-        <x:v>2026-10-09T06:36:40.167Z</x:v>
+        <x:v>2026-10-09T08:38:46.002Z</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="357" customHeight="1">
@@ -4202,7 +4191,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M38" s="14" t="d">
-        <x:v>2026-10-09T06:36:44.265Z</x:v>
+        <x:v>2026-10-09T08:38:50.113Z</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="546" customHeight="1">
@@ -4281,78 +4270,120 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M39" s="14" t="d">
-        <x:v>2026-10-09T06:36:47.311Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="378" customHeight="1">
+        <x:v>2026-10-09T08:38:52.944Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="1050" customHeight="1">
       <x:c r="A40" s="14" t="str">
         <x:v>M39</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
-        <x:v>R04,R07</x:v>
+        <x:v>R02,R04,R05,R10</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>Keyboard, desktop zoom, numeric alignment and saving feedback</x:v>
+        <x:v>Overview visibility before and after Employee starts a task</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>Fresh isolated PostgreSQL test database seeded with Admin, Neha/Arjun Managers, Asha/Ravi Employees, inactive Meera and unassigned Dev. Four projects include empty, unfinished and completed work. Local Chromium at 1440×900, DEBUG=False, source static assets. Use your own record IDs for human retesting. Native browser menu zoom must be tested by a human. Automated reflow uses a 720x450 CSS viewport at 2x density. Saving feedback inspection temporarily prevents navigation in the test browser.</x:v>
+        <x:v>Fresh isolated PostgreSQL test database seeded with Admin, Neha/Arjun Managers, Asha/Ravi Employees, inactive Meera and unassigned Dev. Four projects include empty, unfinished and completed work. Local Chromium at 1440×900, DEBUG=False, source static assets. Use your own record IDs for human retesting.</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
         <x:v>1. GET /login/: 200 (expected 200)
-2. Fill Login identifier = asha@demo.local
+2. Fill Login identifier = neha@demo.local
 3. Fill Password = [password omitted]
 4. Click Sign in
-5. Browser sign-in as asha; Overview displayed
-6. GET /tasks/462/: 200 (expected 200)
-7. Fill Work date = 2026-10-09
-8. Fill Hours = 1
-9. Fill Minutes = 30
-10. Fill Work note = QA40 work
-11. Fill Minutes = 1.5
-12. Click Log time
-13. GET /tasks/462/: 200 (expected 200)
-14. Fill Work date = 2026-10-09
-15. Fill Hours = 1
-16. Fill Minutes = 30
-17. Fill Work note = Single browser submit
-18. Click Log time</x:v>
+5. Browser sign-in as neha; Overview displayed
+6. POST /api/projects/ with JSON {"name":"Overview workflow project","start_date":"2026-10-09","end_date":"2026-10-09"}
+7. POST /api/projects/161/memberships/ with JSON {"employee_id":272}
+8. POST /api/tasks/ with JSON {"project_id":161,"title":"Overview workflow task","assignee_id":272}
+9. GET /login/: 200 (expected 200)
+10. Fill Login identifier = neha@demo.local
+11. Fill Password = [password omitted]
+12. Click Sign in
+13. Browser sign-in as neha; Overview displayed
+14. GET /: 200 (expected 200)
+15. GET /api/overview/ with JSON {}
+16. GET /api/overview/: 200 (expected 200)
+17. GET /login/: 200 (expected 200)
+18. Fill Login identifier = admin@demo.local
+19. Fill Password = [password omitted]
+20. Click Sign in
+21. Browser sign-in as admin; Overview displayed
+22. GET /: 200 (expected 200)
+23. GET /api/overview/ with JSON {}
+24. GET /api/overview/: 200 (expected 200)
+25. GET /login/: 200 (expected 200)
+26. Fill Login identifier = asha@demo.local
+27. Fill Password = [password omitted]
+28. Click Sign in
+29. Browser sign-in as asha; Overview displayed
+30. GET /: 200 (expected 200)
+31. GET /tasks/474/: 200 (expected 200)
+32. Click Start task
+33. GET /login/: 200 (expected 200)
+34. Fill Login identifier = neha@demo.local
+35. Fill Password = [password omitted]
+36. Click Sign in
+37. Browser sign-in as neha; Overview displayed
+38. GET /: 200 (expected 200)
+39. GET /login/: 200 (expected 200)
+40. Fill Login identifier = admin@demo.local
+41. Fill Password = [password omitted]
+42. Click Sign in
+43. Browser sign-in as admin; Overview displayed
+44. GET /: 200 (expected 200)
+45. GET /login/: 200 (expected 200)
+46. Fill Login identifier = arjun@demo.local
+47. Fill Password = [password omitted]
+48. Click Sign in
+49. Browser sign-in as arjun; Overview displayed
+50. GET /: 200 (expected 200)</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
-        <x:v>Fill Login identifier = asha@demo.local
-Fill Password = [password omitted]
-Fill Work date = 2026-10-09
-Fill Hours = 1
-Fill Minutes = 30
-Fill Work note = QA40 work
-Fill Minutes = 1.5
-Fill Work date = 2026-10-09
-Fill Hours = 1
-Fill Minutes = 30
-Fill Work note = Single browser submit</x:v>
+        <x:v>Fill Login identifier = neha@demo.local
+Fill Password = [password omitted]
+POST /api/projects/ {"name":"Overview workflow project","start_date":"2026-10-09","end_date":"2026-10-09"}
+POST /api/projects/161/memberships/ {"employee_id":272}
+POST /api/tasks/ {"project_id":161,"title":"Overview workflow task","assignee_id":272}
+Fill Login identifier = neha@demo.local
+Fill Password = [password omitted]
+GET /api/overview/ {}
+Fill Login identifier = admin@demo.local
+Fill Password = [password omitted]
+GET /api/overview/ {}
+Fill Login identifier = asha@demo.local
+Fill Password = [password omitted]
+Fill Login identifier = neha@demo.local
+Fill Password = [password omitted]
+Fill Login identifier = admin@demo.local
+Fill Password = [password omitted]
+Fill Login identifier = arjun@demo.local
+Fill Password = [password omitted]</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>Controls reachable with visible focus, readable at 200%, and one save.</x:v>
+        <x:v>Admin/Manager totals include the project; TODO task appears in Work in progress only after Start task; Employee sees own TODO work; foreign Manager excluded.</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
-        <x:v>Keyboard focus has visible outline
-Zoom-equivalent viewport has no page-level horizontal overflow
-Minutes has associated helper text
-Submit marks form busy and shows saving feedback
-Disabled button ignores a second click
-One entry saved through browser submission
-Time durations are right aligned
-Native browser 200% zoom and human usability assessment not executed. Zoom-equivalent reflow, keyboard and saving checks executed.</x:v>
+        <x:v>neha: TODO task excluded from Work in progress
+neha: new project included in summary
+admin: TODO task excluded from Work in progress
+admin: new project included in summary
+Employee Overview includes own TODO task
+Employee Start task button persists IN_PROGRESS
+neha: started task and project visible in Work in progress
+admin: started task and project visible in Work in progress
+Foreign Manager cannot see the task</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
-        <x:v>BLOCKED</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="J40" s="14" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="K40" s="14" t="str">
-        <x:v>docs/evidence/qa40/M39-keyboard-error-focus.png
-docs/evidence/qa40/M39-200-percent-viewport-equivalent.png
-docs/evidence/qa40/M39-saving-feedback.png
+        <x:v>docs/evidence/qa40/M39-neha-before-start.png
+docs/evidence/qa40/M39-admin-before-start.png
+docs/evidence/qa40/M39-neha-after-start.png
+docs/evidence/qa40/M39-admin-after-start.png
 docs/evidence/qa40/M39-final.png
 docs/evidence/qa40/M39.json</x:v>
       </x:c>
@@ -4360,7 +4391,7 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M40" s="14" t="d">
-        <x:v>2026-10-09T06:36:50.813Z</x:v>
+        <x:v>2026-10-09T08:38:56.455Z</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="210" customHeight="1">
@@ -4382,20 +4413,20 @@
 3. Fill Password = [password omitted]
 4. Click Sign in
 5. Browser sign-in as neha; Overview displayed
-6. DELETE /api/projects/161/ with JSON {}
-7. DELETE /api/tasks/474/ with JSON {}
-8. DELETE /api/tasks/478/ with JSON {}
-9. DELETE /api/projects/163/ with JSON {}
-10. DELETE /api/tasks/476/ with JSON {}</x:v>
+6. DELETE /api/projects/162/ with JSON {}
+7. DELETE /api/tasks/475/ with JSON {}
+8. DELETE /api/tasks/479/ with JSON {}
+9. DELETE /api/projects/164/ with JSON {}
+10. DELETE /api/tasks/477/ with JSON {}</x:v>
       </x:c>
       <x:c r="F41" s="14" t="str">
         <x:v>Fill Login identifier = neha@demo.local
 Fill Password = [password omitted]
-DELETE /api/projects/161/ {}
-DELETE /api/tasks/474/ {}
-DELETE /api/tasks/478/ {}
-DELETE /api/projects/163/ {}
-DELETE /api/tasks/476/ {}</x:v>
+DELETE /api/projects/162/ {}
+DELETE /api/tasks/475/ {}
+DELETE /api/tasks/479/ {}
+DELETE /api/projects/164/ {}
+DELETE /api/tasks/477/ {}</x:v>
       </x:c>
       <x:c r="G41" s="14" t="str">
         <x:v>Dependent work protected; empty projects and tasks without history removable.</x:v>
@@ -4418,13 +4449,13 @@
         <x:v>Agent-executed Chromium browser/HTTP checks with PostgreSQL readback</x:v>
       </x:c>
       <x:c r="M41" s="14" t="d">
-        <x:v>2026-10-09T06:36:54.387Z</x:v>
+        <x:v>2026-10-09T08:39:01.829Z</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2e94d1374fb49c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d3e649d99c54879"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>